<commit_message>
🚧 wip: RoomManager 까지 완료
</commit_message>
<xml_diff>
--- a/Server/Common/GameDatasheet/Original_Map.xlsx
+++ b/Server/Common/GameDatasheet/Original_Map.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zmwps\Desktop\Project_MMORPG\Server\Common\GameDatasheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEA16F3D-8739-4637-8B88-7FCBD75E0057}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AC711A2-80D6-4150-8D3B-99CFE3CE0139}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" xr2:uid="{FDA0E9BE-2965-48E7-917D-7535984AEDF4}"/>
   </bookViews>
@@ -93,7 +93,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="34">
   <si>
     <t>BOTH</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -139,10 +139,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>min_monster_count</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>SERVER</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -195,40 +191,52 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>respawn_period</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>summon_count</t>
+    <t>[]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>center_pos</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{"pos_x" : -10000, "pos_y": 10000, "pos_z": 0}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{"pos_x" : -10000, "pos_y": 0, "pos_z": 0}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>{"pos_x" : -10000, "pos_y": -10000, "pos_z": 0}</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>monster_respawn_time</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>{"lists": [
-{"portal_id": 21, "type": "room", "src": {"pos_x": -7750, "pos_y": 10000, "pos_z": 0}, "dst": {"pos_x": -1000, "pos_y": 1000, "pos_z": 0}}
+{"portal_id": 11, "type": "room", "src": {"pos_x": -1200, "pos_y": 1000, "pos_z": 0}, "dst": {"template_id": 20, "pos_x": -7750, "pos_y": 10000, "pos_z": 0}}, 
+{"portal_id": 12, "type": "room", "src": {"pos_x": -1200, "pos_y": 0, "pos_z": 0}, "dst": {"template_id": 30, "pos_x": -7750, "pos_y": 0, "pos_z": 0}}, 
+{"portal_id": 13, "type": "room", "src": {"pos_x": -1200, "pos_y": -1000, "pos_z": 0}, "dst": {"template_id": 40, "pos_x": -7750, "pos_y": -10000, "pos_z": 0}}
 ]}</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>{"lists": [
-{"portal_id": 31, "type": "room", "src": {"pos_x": -7750, "pos_y": 0, "pos_z": 0}, "dst": {"pos_x": -1000, "pos_y": 0, "pos_z": 0}}
+{"portal_id": 21, "type": "room", "src": {"pos_x": -7750, "pos_y": 10000, "pos_z": 0}, "dst": {"template_id": 10, "pos_x": -1000, "pos_y": 1000, "pos_z": 0}}
 ]}</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>{"lists": [
-{"portal_id": 41, "type": "room", "src": {"pos_x": -7750, "pos_y": -10000, "pos_z": 0}, "dst": {"pos_x": -1000, "pos_y": -1000, "pos_z": 0}}
+{"portal_id": 31, "type": "room", "src": {"pos_x": -7750, "pos_y": 0, "pos_z": 0}, "dst": {"template_id": 10, "pos_x": -1000, "pos_y": 0, "pos_z": 0}}
 ]}</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>[]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>{"lists": [
-{"portal_id": 11, "type": "room", "src": {"pos_x": -1200, "pos_y": 1000, "pos_z": 0}, "dst": {"pos_x": -7750, "pos_y": 10000, "pos_z": 0}}, 
-{"portal_id": 12, "type": "room", "src": {"pos_x": -1200, "pos_y": 0, "pos_z": 0}, "dst": {"pos_x": -7750, "pos_y": 0, "pos_z": 0}}, 
-{"portal_id": 13, "type": "room", "src": {"pos_x": -1200, "pos_y": -1000, "pos_z": 0}, "dst": {"pos_x": -7750, "pos_y": -10000, "pos_z": 0}}
+{"portal_id": 41, "type": "room", "src": {"pos_x": -7750, "pos_y": -10000, "pos_z": 0}, "dst": {"template_id": 10, "pos_x": -1000, "pos_y": -1000, "pos_z": 0}}
 ]}</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -612,15 +620,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82845201-2628-4823-B6D1-8A4642A35A02}">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="8" max="8" width="13.59765625" customWidth="1"/>
+    <col min="9" max="9" width="13.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B1" t="s">
         <v>3</v>
@@ -629,37 +637,34 @@
         <v>8</v>
       </c>
       <c r="D1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H1" t="s">
         <v>22</v>
       </c>
-      <c r="E1" t="s">
-        <v>20</v>
-      </c>
-      <c r="F1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>23</v>
       </c>
-      <c r="H1" t="s">
-        <v>24</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="K1" t="s">
-        <v>11</v>
-      </c>
       <c r="L1" t="s">
-        <v>25</v>
-      </c>
-      <c r="M1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -673,34 +678,31 @@
         <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="K2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="L2" t="s">
-        <v>12</v>
-      </c>
-      <c r="M2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>10</v>
       </c>
@@ -713,61 +715,61 @@
       <c r="D3" t="s">
         <v>2</v>
       </c>
-      <c r="E3">
-        <v>1500</v>
+      <c r="E3" t="s">
+        <v>16</v>
       </c>
       <c r="F3">
         <v>1500</v>
       </c>
-      <c r="G3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="I3" t="s">
+      <c r="G3">
+        <v>1500</v>
+      </c>
+      <c r="H3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="1" t="s">
         <v>30</v>
       </c>
+      <c r="J3" t="s">
+        <v>24</v>
+      </c>
     </row>
-    <row r="4" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4">
         <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D4" t="s">
         <v>1</v>
       </c>
-      <c r="E4">
-        <v>2500</v>
+      <c r="E4" t="s">
+        <v>26</v>
       </c>
       <c r="F4">
         <v>2500</v>
       </c>
-      <c r="H4" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="I4" t="s">
-        <v>14</v>
-      </c>
-      <c r="J4">
+      <c r="G4">
+        <v>2500</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="J4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K4">
         <v>20</v>
-      </c>
-      <c r="K4">
-        <v>5</v>
       </c>
       <c r="L4">
         <v>10</v>
       </c>
-      <c r="M4">
-        <v>3</v>
-      </c>
     </row>
-    <row r="5" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>30</v>
       </c>
@@ -775,37 +777,34 @@
         <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D5" t="s">
         <v>1</v>
       </c>
-      <c r="E5">
-        <v>2500</v>
+      <c r="E5" t="s">
+        <v>27</v>
       </c>
       <c r="F5">
         <v>2500</v>
       </c>
-      <c r="H5" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="I5" t="s">
-        <v>15</v>
-      </c>
-      <c r="J5">
+      <c r="G5">
+        <v>2500</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="J5" t="s">
+        <v>14</v>
+      </c>
+      <c r="K5">
         <v>20</v>
-      </c>
-      <c r="K5">
-        <v>5</v>
       </c>
       <c r="L5">
         <v>10</v>
       </c>
-      <c r="M5">
-        <v>3</v>
-      </c>
     </row>
-    <row r="6" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6">
         <v>40</v>
       </c>
@@ -813,34 +812,31 @@
         <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D6" t="s">
         <v>1</v>
       </c>
-      <c r="E6">
-        <v>2500</v>
+      <c r="E6" t="s">
+        <v>28</v>
       </c>
       <c r="F6">
         <v>2500</v>
       </c>
-      <c r="H6" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="I6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J6">
+      <c r="G6">
+        <v>2500</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="J6" t="s">
+        <v>15</v>
+      </c>
+      <c r="K6">
         <v>20</v>
-      </c>
-      <c r="K6">
-        <v>5</v>
       </c>
       <c r="L6">
         <v>10</v>
-      </c>
-      <c r="M6">
-        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>